<commit_message>
Fix application status remarks error
</commit_message>
<xml_diff>
--- a/acz_applications.xlsx
+++ b/acz_applications.xlsx
@@ -509,14 +509,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Submitted</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-06-20 13:50:11.122069+00:00</t>
+          <t>2026-06-28 07:01:18.162070+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add admin button and bulk status update
</commit_message>
<xml_diff>
--- a/acz_applications.xlsx
+++ b/acz_applications.xlsx
@@ -509,14 +509,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Submitted</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-06-28 07:01:18.162070+00:00</t>
+          <t>2026-06-28 07:27:32.227356+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add payment and receipt system
</commit_message>
<xml_diff>
--- a/acz_applications.xlsx
+++ b/acz_applications.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,11 +512,56 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>2026-06-28 07:27:32.227356+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Madhu Kumari</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>547854262147</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2479654780</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NEW ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>R355416846</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-06-30 13:43:55.654868+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update homepage design and notice board
</commit_message>
<xml_diff>
--- a/acz_applications.xlsx
+++ b/acz_applications.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,11 +557,101 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>2026-06-30 13:43:55.654868+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MANOJ KUMAR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>628788333412</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3287883334</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NEW ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>R355416846</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-07-01 04:25:33.613956+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MANOJ KUMAR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>628788333412</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3287883334</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PRINT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>32464654646</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-07-01 04:27:22.149487+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer login preloader and application UI
</commit_message>
<xml_diff>
--- a/acz_applications.xlsx
+++ b/acz_applications.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,12 +554,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
+          <t>In Process</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-06-30 13:43:55.654868+00:00</t>
+          <t>2026-07-03 14:58:04.064221+00:00</t>
         </is>
       </c>
     </row>
@@ -647,11 +649,59 @@
           <t>Submitted</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-01 04:27:22.149487+00:00</t>
+          <t>2026-07-02 08:35:10.759007+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MANOJ KUMAR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>628788333412</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3287883334</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PRINT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>518528592</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:43:54.330986+00:00</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:44:18.579534+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>